<commit_message>
ci: add GitHub Action for Google Drive sync
</commit_message>
<xml_diff>
--- a/debug/Engine_Validation_Report.xlsx
+++ b/debug/Engine_Validation_Report.xlsx
@@ -587,13 +587,13 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D2" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E2" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="3">
@@ -604,13 +604,13 @@
         <v>0.01666666666666667</v>
       </c>
       <c r="C3" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D3" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E3" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="4">
@@ -621,13 +621,13 @@
         <v>0.03333333333333333</v>
       </c>
       <c r="C4" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D4" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E4" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="5">
@@ -638,13 +638,13 @@
         <v>0.05</v>
       </c>
       <c r="C5" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E5" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="6">
@@ -655,13 +655,13 @@
         <v>0.06666666666666667</v>
       </c>
       <c r="C6" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E6" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="7">
@@ -672,13 +672,13 @@
         <v>0.08333333333333333</v>
       </c>
       <c r="C7" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E7" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="8">
@@ -689,13 +689,13 @@
         <v>0.09999999999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E8" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="9">
@@ -706,13 +706,13 @@
         <v>0.1166666666666667</v>
       </c>
       <c r="C9" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D9" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E9" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="10">
@@ -723,13 +723,13 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="C10" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E10" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="11">
@@ -740,13 +740,13 @@
         <v>0.15</v>
       </c>
       <c r="C11" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E11" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="12">
@@ -757,13 +757,13 @@
         <v>0.1666666666666667</v>
       </c>
       <c r="C12" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D12" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E12" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="13">
@@ -774,13 +774,13 @@
         <v>0.1833333333333333</v>
       </c>
       <c r="C13" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E13" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="14">
@@ -791,13 +791,13 @@
         <v>0.2</v>
       </c>
       <c r="C14" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D14" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E14" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="15">
@@ -808,13 +808,13 @@
         <v>0.2166666666666666</v>
       </c>
       <c r="C15" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E15" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="16">
@@ -825,13 +825,13 @@
         <v>0.2333333333333333</v>
       </c>
       <c r="C16" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E16" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="17">
@@ -842,13 +842,13 @@
         <v>0.25</v>
       </c>
       <c r="C17" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D17" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E17" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="18">
@@ -859,13 +859,13 @@
         <v>0.2666666666666667</v>
       </c>
       <c r="C18" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D18" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E18" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="19">
@@ -876,13 +876,13 @@
         <v>0.2833333333333333</v>
       </c>
       <c r="C19" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D19" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E19" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="20">
@@ -893,13 +893,13 @@
         <v>0.3</v>
       </c>
       <c r="C20" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D20" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E20" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="21">
@@ -910,13 +910,13 @@
         <v>0.3166666666666667</v>
       </c>
       <c r="C21" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D21" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E21" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="22">
@@ -927,13 +927,13 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="C22" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D22" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E22" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="23">
@@ -944,13 +944,13 @@
         <v>0.35</v>
       </c>
       <c r="C23" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D23" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E23" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="24">
@@ -961,13 +961,13 @@
         <v>0.3666666666666666</v>
       </c>
       <c r="C24" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D24" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E24" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="25">
@@ -978,13 +978,13 @@
         <v>0.3833333333333333</v>
       </c>
       <c r="C25" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D25" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E25" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="26">
@@ -995,13 +995,13 @@
         <v>0.4</v>
       </c>
       <c r="C26" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D26" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E26" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="27">
@@ -1012,13 +1012,13 @@
         <v>0.4166666666666666</v>
       </c>
       <c r="C27" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D27" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E27" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="28">
@@ -1029,13 +1029,13 @@
         <v>0.4333333333333333</v>
       </c>
       <c r="C28" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D28" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E28" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="29">
@@ -1046,13 +1046,13 @@
         <v>0.45</v>
       </c>
       <c r="C29" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D29" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E29" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="30">
@@ -1063,13 +1063,13 @@
         <v>0.4666666666666666</v>
       </c>
       <c r="C30" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D30" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E30" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="31">
@@ -1080,13 +1080,13 @@
         <v>0.4833333333333333</v>
       </c>
       <c r="C31" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D31" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E31" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="32">
@@ -1097,13 +1097,13 @@
         <v>0.4999999999999999</v>
       </c>
       <c r="C32" t="n">
-        <v>314</v>
+        <v>467.9999999999999</v>
       </c>
       <c r="D32" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E32" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="33">
@@ -1114,13 +1114,13 @@
         <v>0.5166666666666666</v>
       </c>
       <c r="C33" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D33" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E33" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="34">
@@ -1131,13 +1131,13 @@
         <v>0.5333333333333333</v>
       </c>
       <c r="C34" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D34" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E34" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="35">
@@ -1148,13 +1148,13 @@
         <v>0.55</v>
       </c>
       <c r="C35" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D35" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E35" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="36">
@@ -1165,13 +1165,13 @@
         <v>0.5666666666666668</v>
       </c>
       <c r="C36" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D36" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E36" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="37">
@@ -1182,13 +1182,13 @@
         <v>0.5833333333333335</v>
       </c>
       <c r="C37" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D37" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E37" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="38">
@@ -1199,13 +1199,13 @@
         <v>0.6000000000000002</v>
       </c>
       <c r="C38" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D38" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E38" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="39">
@@ -1216,13 +1216,13 @@
         <v>0.6166666666666669</v>
       </c>
       <c r="C39" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D39" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E39" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="40">
@@ -1233,13 +1233,13 @@
         <v>0.6333333333333336</v>
       </c>
       <c r="C40" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D40" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E40" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="41">
@@ -1250,13 +1250,13 @@
         <v>0.6500000000000004</v>
       </c>
       <c r="C41" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D41" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E41" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="42">
@@ -1267,13 +1267,13 @@
         <v>0.6666666666666671</v>
       </c>
       <c r="C42" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D42" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E42" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="43">
@@ -1284,13 +1284,13 @@
         <v>0.6833333333333338</v>
       </c>
       <c r="C43" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D43" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E43" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="44">
@@ -1301,13 +1301,13 @@
         <v>0.7000000000000005</v>
       </c>
       <c r="C44" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D44" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E44" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="45">
@@ -1318,13 +1318,13 @@
         <v>0.7166666666666672</v>
       </c>
       <c r="C45" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D45" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E45" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="46">
@@ -1335,13 +1335,13 @@
         <v>0.7333333333333339</v>
       </c>
       <c r="C46" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D46" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E46" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="47">
@@ -1352,13 +1352,13 @@
         <v>0.7500000000000007</v>
       </c>
       <c r="C47" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D47" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E47" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="48">
@@ -1369,13 +1369,13 @@
         <v>0.7666666666666674</v>
       </c>
       <c r="C48" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D48" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E48" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="49">
@@ -1386,13 +1386,13 @@
         <v>0.7833333333333341</v>
       </c>
       <c r="C49" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D49" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E49" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="50">
@@ -1403,13 +1403,13 @@
         <v>0.8000000000000008</v>
       </c>
       <c r="C50" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D50" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E50" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="51">
@@ -1420,13 +1420,13 @@
         <v>0.8166666666666675</v>
       </c>
       <c r="C51" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D51" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E51" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="52">
@@ -1437,13 +1437,13 @@
         <v>0.8333333333333343</v>
       </c>
       <c r="C52" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D52" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E52" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="53">
@@ -1454,13 +1454,13 @@
         <v>0.850000000000001</v>
       </c>
       <c r="C53" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D53" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E53" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="54">
@@ -1471,13 +1471,13 @@
         <v>0.8666666666666677</v>
       </c>
       <c r="C54" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D54" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E54" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="55">
@@ -1488,13 +1488,13 @@
         <v>0.8833333333333344</v>
       </c>
       <c r="C55" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D55" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E55" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="56">
@@ -1505,13 +1505,13 @@
         <v>0.9000000000000011</v>
       </c>
       <c r="C56" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D56" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E56" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="57">
@@ -1522,13 +1522,13 @@
         <v>0.9166666666666679</v>
       </c>
       <c r="C57" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D57" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E57" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="58">
@@ -1539,13 +1539,13 @@
         <v>0.9333333333333346</v>
       </c>
       <c r="C58" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D58" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E58" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="59">
@@ -1556,13 +1556,13 @@
         <v>0.9500000000000013</v>
       </c>
       <c r="C59" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D59" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E59" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="60">
@@ -1573,13 +1573,13 @@
         <v>0.966666666666668</v>
       </c>
       <c r="C60" t="n">
-        <v>314</v>
+        <v>468</v>
       </c>
       <c r="D60" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E60" t="n">
-        <v>251.043</v>
+        <v>14.13594</v>
       </c>
     </row>
     <row r="61">
@@ -1590,13 +1590,13 @@
         <v>0.9833333333333347</v>
       </c>
       <c r="C61" t="n">
-        <v>314</v>
+        <v>467.9999999999609</v>
       </c>
       <c r="D61" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E61" t="n">
-        <v>251.043</v>
+        <v>14.13593999999882</v>
       </c>
     </row>
     <row r="62">
@@ -1607,13 +1607,13 @@
         <v>1</v>
       </c>
       <c r="C62" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D62" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E62" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="63">
@@ -1624,13 +1624,13 @@
         <v>0.9833333333333333</v>
       </c>
       <c r="C63" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D63" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E63" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="64">
@@ -1641,13 +1641,13 @@
         <v>0.9666666666666666</v>
       </c>
       <c r="C64" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D64" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E64" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="65">
@@ -1658,13 +1658,13 @@
         <v>0.9499999999999998</v>
       </c>
       <c r="C65" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D65" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E65" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="66">
@@ -1675,13 +1675,13 @@
         <v>0.9333333333333331</v>
       </c>
       <c r="C66" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D66" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E66" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="67">
@@ -1692,13 +1692,13 @@
         <v>0.9166666666666664</v>
       </c>
       <c r="C67" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D67" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E67" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="68">
@@ -1709,13 +1709,13 @@
         <v>0.8999999999999997</v>
       </c>
       <c r="C68" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D68" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E68" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="69">
@@ -1726,13 +1726,13 @@
         <v>0.883333333333333</v>
       </c>
       <c r="C69" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D69" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E69" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="70">
@@ -1743,13 +1743,13 @@
         <v>0.8666666666666663</v>
       </c>
       <c r="C70" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D70" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E70" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="71">
@@ -1760,13 +1760,13 @@
         <v>0.8499999999999995</v>
       </c>
       <c r="C71" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D71" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E71" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="72">
@@ -1777,13 +1777,13 @@
         <v>0.8333333333333328</v>
       </c>
       <c r="C72" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D72" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E72" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="73">
@@ -1794,13 +1794,13 @@
         <v>0.8166666666666661</v>
       </c>
       <c r="C73" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D73" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E73" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="74">
@@ -1811,13 +1811,13 @@
         <v>0.7999999999999994</v>
       </c>
       <c r="C74" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D74" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E74" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="75">
@@ -1828,13 +1828,13 @@
         <v>0.7833333333333327</v>
       </c>
       <c r="C75" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D75" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E75" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="76">
@@ -1845,13 +1845,13 @@
         <v>0.7666666666666659</v>
       </c>
       <c r="C76" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D76" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E76" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="77">
@@ -1862,13 +1862,13 @@
         <v>0.7499999999999992</v>
       </c>
       <c r="C77" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D77" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E77" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="78">
@@ -1879,13 +1879,13 @@
         <v>0.7333333333333325</v>
       </c>
       <c r="C78" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D78" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E78" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="79">
@@ -1896,13 +1896,13 @@
         <v>0.7166666666666658</v>
       </c>
       <c r="C79" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D79" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E79" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="80">
@@ -1913,13 +1913,13 @@
         <v>0.6999999999999991</v>
       </c>
       <c r="C80" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D80" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E80" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="81">
@@ -1930,13 +1930,13 @@
         <v>0.6833333333333323</v>
       </c>
       <c r="C81" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D81" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E81" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="82">
@@ -1947,13 +1947,13 @@
         <v>0.6666666666666656</v>
       </c>
       <c r="C82" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D82" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E82" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="83">
@@ -1964,13 +1964,13 @@
         <v>0.6499999999999989</v>
       </c>
       <c r="C83" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D83" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E83" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="84">
@@ -1981,13 +1981,13 @@
         <v>0.6333333333333322</v>
       </c>
       <c r="C84" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D84" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E84" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="85">
@@ -1998,13 +1998,13 @@
         <v>0.6166666666666655</v>
       </c>
       <c r="C85" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D85" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E85" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="86">
@@ -2015,13 +2015,13 @@
         <v>0.5999999999999988</v>
       </c>
       <c r="C86" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D86" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E86" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="87">
@@ -2032,13 +2032,13 @@
         <v>0.583333333333332</v>
       </c>
       <c r="C87" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D87" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E87" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="88">
@@ -2049,13 +2049,13 @@
         <v>0.5666666666666653</v>
       </c>
       <c r="C88" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D88" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E88" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="89">
@@ -2066,13 +2066,13 @@
         <v>0.5499999999999986</v>
       </c>
       <c r="C89" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D89" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E89" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="90">
@@ -2083,13 +2083,13 @@
         <v>0.5333333333333319</v>
       </c>
       <c r="C90" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D90" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E90" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="91">
@@ -2100,13 +2100,13 @@
         <v>0.5166666666666652</v>
       </c>
       <c r="C91" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D91" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E91" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="92">
@@ -2117,13 +2117,13 @@
         <v>0.4999999999999985</v>
       </c>
       <c r="C92" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D92" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E92" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="93">
@@ -2134,13 +2134,13 @@
         <v>0.4833333333333318</v>
       </c>
       <c r="C93" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D93" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E93" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="94">
@@ -2151,13 +2151,13 @@
         <v>0.4666666666666652</v>
       </c>
       <c r="C94" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D94" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E94" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="95">
@@ -2168,13 +2168,13 @@
         <v>0.4499999999999985</v>
       </c>
       <c r="C95" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D95" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E95" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="96">
@@ -2185,13 +2185,13 @@
         <v>0.4333333333333318</v>
       </c>
       <c r="C96" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D96" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E96" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="97">
@@ -2202,13 +2202,13 @@
         <v>0.4166666666666652</v>
       </c>
       <c r="C97" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D97" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E97" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="98">
@@ -2219,13 +2219,13 @@
         <v>0.3999999999999985</v>
       </c>
       <c r="C98" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D98" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E98" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="99">
@@ -2236,13 +2236,13 @@
         <v>0.3833333333333319</v>
       </c>
       <c r="C99" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D99" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E99" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="100">
@@ -2253,13 +2253,13 @@
         <v>0.3666666666666652</v>
       </c>
       <c r="C100" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D100" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E100" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="101">
@@ -2270,13 +2270,13 @@
         <v>0.3499999999999985</v>
       </c>
       <c r="C101" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D101" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E101" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="102">
@@ -2287,13 +2287,13 @@
         <v>0.3333333333333319</v>
       </c>
       <c r="C102" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D102" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E102" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="103">
@@ -2304,13 +2304,13 @@
         <v>0.3166666666666652</v>
       </c>
       <c r="C103" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D103" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E103" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="104">
@@ -2321,13 +2321,13 @@
         <v>0.2999999999999985</v>
       </c>
       <c r="C104" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D104" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E104" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="105">
@@ -2338,13 +2338,13 @@
         <v>0.2833333333333319</v>
       </c>
       <c r="C105" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D105" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E105" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="106">
@@ -2355,13 +2355,13 @@
         <v>0.2666666666666652</v>
       </c>
       <c r="C106" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D106" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E106" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="107">
@@ -2372,13 +2372,13 @@
         <v>0.2499999999999986</v>
       </c>
       <c r="C107" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D107" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E107" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="108">
@@ -2389,13 +2389,13 @@
         <v>0.2333333333333319</v>
       </c>
       <c r="C108" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D108" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E108" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="109">
@@ -2406,13 +2406,13 @@
         <v>0.2166666666666652</v>
       </c>
       <c r="C109" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D109" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E109" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="110">
@@ -2423,13 +2423,13 @@
         <v>0.1999999999999986</v>
       </c>
       <c r="C110" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D110" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E110" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="111">
@@ -2440,13 +2440,13 @@
         <v>0.1833333333333319</v>
       </c>
       <c r="C111" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D111" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E111" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="112">
@@ -2457,13 +2457,13 @@
         <v>0.1666666666666652</v>
       </c>
       <c r="C112" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D112" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E112" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="113">
@@ -2474,13 +2474,13 @@
         <v>0.1499999999999986</v>
       </c>
       <c r="C113" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D113" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E113" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="114">
@@ -2491,13 +2491,13 @@
         <v>0.1333333333333319</v>
       </c>
       <c r="C114" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D114" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E114" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="115">
@@ -2508,13 +2508,13 @@
         <v>0.1166666666666653</v>
       </c>
       <c r="C115" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D115" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E115" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="116">
@@ -2525,13 +2525,13 @@
         <v>0.09999999999999859</v>
       </c>
       <c r="C116" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D116" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E116" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="117">
@@ -2542,13 +2542,13 @@
         <v>0.08333333333333193</v>
       </c>
       <c r="C117" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D117" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E117" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="118">
@@ -2559,13 +2559,13 @@
         <v>0.06666666666666526</v>
       </c>
       <c r="C118" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D118" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E118" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="119">
@@ -2576,13 +2576,13 @@
         <v>0.0499999999999986</v>
       </c>
       <c r="C119" t="n">
-        <v>-314</v>
+        <v>-467.9999999999999</v>
       </c>
       <c r="D119" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E119" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="120">
@@ -2593,13 +2593,13 @@
         <v>0.03333333333333194</v>
       </c>
       <c r="C120" t="n">
-        <v>-314</v>
+        <v>-468</v>
       </c>
       <c r="D120" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E120" t="n">
-        <v>-251.043</v>
+        <v>-14.13594</v>
       </c>
     </row>
     <row r="121">
@@ -2610,13 +2610,13 @@
         <v>0.01666666666666527</v>
       </c>
       <c r="C121" t="n">
-        <v>-314</v>
+        <v>-467.9999999999609</v>
       </c>
       <c r="D121" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E121" t="n">
-        <v>-251.043</v>
+        <v>-14.13593999999882</v>
       </c>
     </row>
   </sheetData>
@@ -2668,13 +2668,13 @@
         <v>0.5</v>
       </c>
       <c r="C2" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D2" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E2" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="3">
@@ -2685,13 +2685,13 @@
         <v>0.5016666666666667</v>
       </c>
       <c r="C3" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D3" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E3" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="4">
@@ -2702,13 +2702,13 @@
         <v>0.5033333333333334</v>
       </c>
       <c r="C4" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D4" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E4" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="5">
@@ -2719,13 +2719,13 @@
         <v>0.5050000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D5" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E5" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="6">
@@ -2736,13 +2736,13 @@
         <v>0.5066666666666668</v>
       </c>
       <c r="C6" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D6" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E6" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="7">
@@ -2753,13 +2753,13 @@
         <v>0.5083333333333335</v>
       </c>
       <c r="C7" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D7" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E7" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="8">
@@ -2770,13 +2770,13 @@
         <v>0.5100000000000002</v>
       </c>
       <c r="C8" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D8" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E8" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="9">
@@ -2787,13 +2787,13 @@
         <v>0.5116666666666669</v>
       </c>
       <c r="C9" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D9" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E9" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="10">
@@ -2804,13 +2804,13 @@
         <v>0.5133333333333336</v>
       </c>
       <c r="C10" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D10" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E10" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="11">
@@ -2821,13 +2821,13 @@
         <v>0.5150000000000003</v>
       </c>
       <c r="C11" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D11" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E11" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="12">
@@ -2838,13 +2838,13 @@
         <v>0.5166666666666671</v>
       </c>
       <c r="C12" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D12" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E12" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="13">
@@ -2855,13 +2855,13 @@
         <v>0.5183333333333338</v>
       </c>
       <c r="C13" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D13" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E13" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="14">
@@ -2872,13 +2872,13 @@
         <v>0.5200000000000005</v>
       </c>
       <c r="C14" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D14" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E14" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="15">
@@ -2889,13 +2889,13 @@
         <v>0.5216666666666672</v>
       </c>
       <c r="C15" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D15" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E15" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="16">
@@ -2906,13 +2906,13 @@
         <v>0.5233333333333339</v>
       </c>
       <c r="C16" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D16" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E16" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="17">
@@ -2923,13 +2923,13 @@
         <v>0.5250000000000006</v>
       </c>
       <c r="C17" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D17" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E17" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="18">
@@ -2940,13 +2940,13 @@
         <v>0.5266666666666673</v>
       </c>
       <c r="C18" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D18" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E18" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="19">
@@ -2957,13 +2957,13 @@
         <v>0.528333333333334</v>
       </c>
       <c r="C19" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D19" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E19" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="20">
@@ -2974,13 +2974,13 @@
         <v>0.5300000000000007</v>
       </c>
       <c r="C20" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D20" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E20" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="21">
@@ -2991,13 +2991,13 @@
         <v>0.5316666666666674</v>
       </c>
       <c r="C21" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D21" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E21" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="22">
@@ -3008,13 +3008,13 @@
         <v>0.5333333333333341</v>
       </c>
       <c r="C22" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D22" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E22" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="23">
@@ -3025,13 +3025,13 @@
         <v>0.5350000000000008</v>
       </c>
       <c r="C23" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D23" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E23" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="24">
@@ -3042,13 +3042,13 @@
         <v>0.5366666666666675</v>
       </c>
       <c r="C24" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D24" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E24" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="25">
@@ -3059,13 +3059,13 @@
         <v>0.5383333333333342</v>
       </c>
       <c r="C25" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D25" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E25" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="26">
@@ -3076,13 +3076,13 @@
         <v>0.5400000000000009</v>
       </c>
       <c r="C26" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D26" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E26" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="27">
@@ -3093,13 +3093,13 @@
         <v>0.5416666666666676</v>
       </c>
       <c r="C27" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D27" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E27" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="28">
@@ -3110,13 +3110,13 @@
         <v>0.5433333333333343</v>
       </c>
       <c r="C28" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D28" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E28" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="29">
@@ -3127,13 +3127,13 @@
         <v>0.545000000000001</v>
       </c>
       <c r="C29" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D29" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E29" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="30">
@@ -3144,13 +3144,13 @@
         <v>0.5466666666666677</v>
       </c>
       <c r="C30" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D30" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E30" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="31">
@@ -3161,13 +3161,13 @@
         <v>0.5483333333333344</v>
       </c>
       <c r="C31" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D31" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E31" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="32">
@@ -3178,13 +3178,13 @@
         <v>0.5500000000000012</v>
       </c>
       <c r="C32" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D32" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E32" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="33">
@@ -3195,13 +3195,13 @@
         <v>0.5516666666666679</v>
       </c>
       <c r="C33" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D33" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E33" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="34">
@@ -3212,13 +3212,13 @@
         <v>0.5533333333333346</v>
       </c>
       <c r="C34" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D34" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E34" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="35">
@@ -3229,13 +3229,13 @@
         <v>0.5550000000000013</v>
       </c>
       <c r="C35" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D35" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E35" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="36">
@@ -3246,13 +3246,13 @@
         <v>0.556666666666668</v>
       </c>
       <c r="C36" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D36" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E36" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="37">
@@ -3263,13 +3263,13 @@
         <v>0.5583333333333347</v>
       </c>
       <c r="C37" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D37" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E37" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="38">
@@ -3280,13 +3280,13 @@
         <v>0.5600000000000014</v>
       </c>
       <c r="C38" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D38" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E38" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="39">
@@ -3297,13 +3297,13 @@
         <v>0.5616666666666681</v>
       </c>
       <c r="C39" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D39" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E39" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="40">
@@ -3314,13 +3314,13 @@
         <v>0.5633333333333348</v>
       </c>
       <c r="C40" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D40" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E40" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="41">
@@ -3331,13 +3331,13 @@
         <v>0.5650000000000015</v>
       </c>
       <c r="C41" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D41" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E41" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="42">
@@ -3348,13 +3348,13 @@
         <v>0.5666666666666682</v>
       </c>
       <c r="C42" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D42" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E42" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="43">
@@ -3365,13 +3365,13 @@
         <v>0.5683333333333349</v>
       </c>
       <c r="C43" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D43" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E43" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="44">
@@ -3382,13 +3382,13 @@
         <v>0.5700000000000016</v>
       </c>
       <c r="C44" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D44" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E44" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="45">
@@ -3399,13 +3399,13 @@
         <v>0.5716666666666683</v>
       </c>
       <c r="C45" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D45" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E45" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="46">
@@ -3416,13 +3416,13 @@
         <v>0.573333333333335</v>
       </c>
       <c r="C46" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D46" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E46" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="47">
@@ -3433,13 +3433,13 @@
         <v>0.5750000000000017</v>
       </c>
       <c r="C47" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D47" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E47" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="48">
@@ -3450,13 +3450,13 @@
         <v>0.5766666666666684</v>
       </c>
       <c r="C48" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D48" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E48" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="49">
@@ -3467,13 +3467,13 @@
         <v>0.5783333333333351</v>
       </c>
       <c r="C49" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D49" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E49" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="50">
@@ -3484,13 +3484,13 @@
         <v>0.5800000000000018</v>
       </c>
       <c r="C50" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D50" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E50" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="51">
@@ -3501,13 +3501,13 @@
         <v>0.5816666666666686</v>
       </c>
       <c r="C51" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D51" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E51" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="52">
@@ -3518,13 +3518,13 @@
         <v>0.5833333333333353</v>
       </c>
       <c r="C52" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D52" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E52" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="53">
@@ -3535,13 +3535,13 @@
         <v>0.585000000000002</v>
       </c>
       <c r="C53" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D53" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E53" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="54">
@@ -3552,13 +3552,13 @@
         <v>0.5866666666666687</v>
       </c>
       <c r="C54" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D54" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E54" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="55">
@@ -3569,13 +3569,13 @@
         <v>0.5883333333333354</v>
       </c>
       <c r="C55" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D55" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E55" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="56">
@@ -3586,13 +3586,13 @@
         <v>0.5900000000000021</v>
       </c>
       <c r="C56" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D56" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E56" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="57">
@@ -3603,13 +3603,13 @@
         <v>0.5916666666666688</v>
       </c>
       <c r="C57" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D57" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E57" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="58">
@@ -3620,13 +3620,13 @@
         <v>0.5933333333333355</v>
       </c>
       <c r="C58" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D58" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E58" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="59">
@@ -3637,13 +3637,13 @@
         <v>0.5950000000000022</v>
       </c>
       <c r="C59" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D59" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E59" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="60">
@@ -3654,13 +3654,13 @@
         <v>0.5966666666666689</v>
       </c>
       <c r="C60" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D60" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E60" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="61">
@@ -3671,13 +3671,13 @@
         <v>0.5983333333333356</v>
       </c>
       <c r="C61" t="n">
-        <v>31.4</v>
+        <v>46.8</v>
       </c>
       <c r="D61" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E61" t="n">
-        <v>25.1043</v>
+        <v>1.413594</v>
       </c>
     </row>
     <row r="62">
@@ -3688,13 +3688,13 @@
         <v>0.6000000000000023</v>
       </c>
       <c r="C62" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D62" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E62" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="63">
@@ -3705,13 +3705,13 @@
         <v>0.5983333333333356</v>
       </c>
       <c r="C63" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D63" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E63" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="64">
@@ -3722,13 +3722,13 @@
         <v>0.5966666666666689</v>
       </c>
       <c r="C64" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D64" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E64" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="65">
@@ -3739,13 +3739,13 @@
         <v>0.5950000000000022</v>
       </c>
       <c r="C65" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D65" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E65" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="66">
@@ -3756,13 +3756,13 @@
         <v>0.5933333333333355</v>
       </c>
       <c r="C66" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D66" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E66" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="67">
@@ -3773,13 +3773,13 @@
         <v>0.5916666666666688</v>
       </c>
       <c r="C67" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D67" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E67" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="68">
@@ -3790,13 +3790,13 @@
         <v>0.5900000000000021</v>
       </c>
       <c r="C68" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D68" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E68" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="69">
@@ -3807,13 +3807,13 @@
         <v>0.5883333333333354</v>
       </c>
       <c r="C69" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D69" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E69" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="70">
@@ -3824,13 +3824,13 @@
         <v>0.5866666666666687</v>
       </c>
       <c r="C70" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D70" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E70" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="71">
@@ -3841,13 +3841,13 @@
         <v>0.585000000000002</v>
       </c>
       <c r="C71" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D71" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E71" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="72">
@@ -3858,13 +3858,13 @@
         <v>0.5833333333333353</v>
       </c>
       <c r="C72" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D72" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E72" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="73">
@@ -3875,13 +3875,13 @@
         <v>0.5816666666666686</v>
       </c>
       <c r="C73" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D73" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E73" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="74">
@@ -3892,13 +3892,13 @@
         <v>0.5800000000000018</v>
       </c>
       <c r="C74" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D74" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E74" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="75">
@@ -3909,13 +3909,13 @@
         <v>0.5783333333333351</v>
       </c>
       <c r="C75" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D75" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E75" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="76">
@@ -3926,13 +3926,13 @@
         <v>0.5766666666666684</v>
       </c>
       <c r="C76" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D76" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E76" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="77">
@@ -3943,13 +3943,13 @@
         <v>0.5750000000000017</v>
       </c>
       <c r="C77" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D77" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E77" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="78">
@@ -3960,13 +3960,13 @@
         <v>0.573333333333335</v>
       </c>
       <c r="C78" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D78" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E78" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="79">
@@ -3977,13 +3977,13 @@
         <v>0.5716666666666683</v>
       </c>
       <c r="C79" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D79" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E79" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="80">
@@ -3994,13 +3994,13 @@
         <v>0.5700000000000016</v>
       </c>
       <c r="C80" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D80" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E80" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="81">
@@ -4011,13 +4011,13 @@
         <v>0.5683333333333349</v>
       </c>
       <c r="C81" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D81" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E81" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="82">
@@ -4028,13 +4028,13 @@
         <v>0.5666666666666682</v>
       </c>
       <c r="C82" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D82" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E82" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="83">
@@ -4045,13 +4045,13 @@
         <v>0.5650000000000015</v>
       </c>
       <c r="C83" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D83" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E83" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="84">
@@ -4062,13 +4062,13 @@
         <v>0.5633333333333348</v>
       </c>
       <c r="C84" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D84" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E84" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="85">
@@ -4079,13 +4079,13 @@
         <v>0.5616666666666681</v>
       </c>
       <c r="C85" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D85" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E85" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="86">
@@ -4096,13 +4096,13 @@
         <v>0.5600000000000014</v>
       </c>
       <c r="C86" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D86" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E86" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="87">
@@ -4113,13 +4113,13 @@
         <v>0.5583333333333347</v>
       </c>
       <c r="C87" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D87" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E87" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="88">
@@ -4130,13 +4130,13 @@
         <v>0.556666666666668</v>
       </c>
       <c r="C88" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D88" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E88" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="89">
@@ -4147,13 +4147,13 @@
         <v>0.5550000000000013</v>
       </c>
       <c r="C89" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D89" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E89" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="90">
@@ -4164,13 +4164,13 @@
         <v>0.5533333333333346</v>
       </c>
       <c r="C90" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D90" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E90" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="91">
@@ -4181,13 +4181,13 @@
         <v>0.5516666666666679</v>
       </c>
       <c r="C91" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D91" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E91" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="92">
@@ -4198,13 +4198,13 @@
         <v>0.5500000000000012</v>
       </c>
       <c r="C92" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D92" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E92" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="93">
@@ -4215,13 +4215,13 @@
         <v>0.5483333333333344</v>
       </c>
       <c r="C93" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D93" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E93" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="94">
@@ -4232,13 +4232,13 @@
         <v>0.5466666666666677</v>
       </c>
       <c r="C94" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D94" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E94" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="95">
@@ -4249,13 +4249,13 @@
         <v>0.545000000000001</v>
       </c>
       <c r="C95" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D95" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E95" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="96">
@@ -4266,13 +4266,13 @@
         <v>0.5433333333333343</v>
       </c>
       <c r="C96" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D96" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E96" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="97">
@@ -4283,13 +4283,13 @@
         <v>0.5416666666666676</v>
       </c>
       <c r="C97" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D97" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E97" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="98">
@@ -4300,13 +4300,13 @@
         <v>0.5400000000000009</v>
       </c>
       <c r="C98" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D98" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E98" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="99">
@@ -4317,13 +4317,13 @@
         <v>0.5383333333333342</v>
       </c>
       <c r="C99" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D99" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E99" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="100">
@@ -4334,13 +4334,13 @@
         <v>0.5366666666666675</v>
       </c>
       <c r="C100" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D100" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E100" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
     <row r="101">
@@ -4351,13 +4351,13 @@
         <v>0.5350000000000008</v>
       </c>
       <c r="C101" t="n">
-        <v>-31.4</v>
+        <v>-46.8</v>
       </c>
       <c r="D101" t="n">
-        <v>799.5</v>
+        <v>30.205</v>
       </c>
       <c r="E101" t="n">
-        <v>-25.1043</v>
+        <v>-1.413594</v>
       </c>
     </row>
   </sheetData>

</xml_diff>